<commit_message>
July 2026 - response values
</commit_message>
<xml_diff>
--- a/Short Adult Version/REACH - SAV_codebook_20May2026.xlsx
+++ b/Short Adult Version/REACH - SAV_codebook_20May2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huntlc/Documents/REACH Website/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huntlc/Documents/REACH Website/NEW July 2026/SAV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334AC223-92AD-4A47-8D4C-F790EB185648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C4321E4-261F-644E-BA7C-74AE0EC26E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="56260" yWindow="660" windowWidth="16700" windowHeight="20940" xr2:uid="{DC13C6BE-47AD-594D-B3E9-96CB9381A8CF}"/>
+    <workbookView xWindow="17840" yWindow="660" windowWidth="16700" windowHeight="20940" xr2:uid="{DC13C6BE-47AD-594D-B3E9-96CB9381A8CF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="289">
   <si>
     <t>Training Instructions</t>
   </si>
@@ -1095,12 +1095,78 @@
   <si>
     <t>0. OTHER ID VARIABLES IN FINAL OUTPUTS (EMA_OUTPUT_FINAL, FLOW_FINAL, EMA_CLEAN)</t>
   </si>
+  <si>
+    <t>Response Values</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>1: 1 (score: 1), 2: 2 (score: 2), 3: 3 (score: 3), 4: 4 (score: 4), 5: 5 (score: 5), 6: 6 (score: 6), 7: 7 (score: 7)</t>
+  </si>
+  <si>
+    <t>Difficulty falling asleep: 0 (score: 1), Awakening too early: 1 (score: 2), Feeling unrefreshed or unrestored despite enough hours of sleep: 2 (score: 3), Nightmares: 3 (score: 4), Other sleep problem: 4 (score: 5), None of the above: 5 (score: 6)</t>
+  </si>
+  <si>
+    <t>Inside: 0 (score: 0), Outside: 1 (score: 1)</t>
+  </si>
+  <si>
+    <t>In your home: 0 (score: 1), In home of relative or friend: 1 (score: 2), At work or in class: 2 (score: 3), In a restaurant/bar or in a store : 3 (score: 4), In a gym or fitness center: 4 (score: 5), In a hospital or doctor’s office : 5 (score: 6), Other place inside: 6 (score: 7)</t>
+  </si>
+  <si>
+    <t>In a public park or garden: 0 (score: 1), In your yard or at home: 1 (score: 2), In your neighborhood: 3 (score: 3), At school: 4 (score: 4), In a vehicle (car, bus…) : 5 (score: 5), In other place outside: 6 (score: 6)</t>
+  </si>
+  <si>
+    <t>No one: 0 (score: 1), A family member: 1 (score: 2), Your romantic partner: 2 (score: 3), Friends: 3 (score: 4), Colleagues or classmates: 4 (score: 5), Strangers: 5 (score: 6), Healthcare provider: 6 (score: 7), Pets: 7 (score: 8)</t>
+  </si>
+  <si>
+    <t>Working or studying: 0 (score: 1), Socializing in person: 1 (score: 2), Using your phone: 2 (score: 3), Watching TV/videos, playing video games, reading: 3 (score: 4), Traveling or commuting: 4 (score: 5), Household chores, shopping: 5 (score: 6), Physical exercise: 6 (score: 7), Eating/drinking: 7 (score: 8), Personal hygiene care: 8 (score: 9), Medical procedure or treatment: 9 (score: 10), Nothing, resting: 10 (score: 11), Other activity: 11 (score: 12)</t>
+  </si>
+  <si>
+    <t>I did not use a computer, tablet, phone or watch TV: 0 (score: 0), Less Than 1 Hour: 1 (score: 1), 1-2 Hours: 2 (score: 2), 2-3 Hours: 3 (score: 3), 3-4 Hours: 4 (score: 4), More Than 4 Hours: 5 (score: 5)</t>
+  </si>
+  <si>
+    <t>Social interactions in-person: 0 (score: 1), Social interactions online/on the phone: 1 (score: 2), Accomplishment/getting things done: 2 (score: 3), Health event/medical care: 3 (score: 4), Learning about or witnessing something upsetting or something heartwarming: 4 (score: 5), Other: 5 (score: 6)</t>
+  </si>
+  <si>
+    <t>Vigorous activities (e.g. running, fast cycling, heavy lifting or digging): 0 (score: 1), Moderate activities (e.g. bicycling, carrying light loads): 1 (score: 2), Light activities (e.g. walking, climbing stairs, routine household chores) : 2 (score: 3), Sedentary activites (e.g. napping, resting, or sitting): 3 (score: 4)</t>
+  </si>
+  <si>
+    <t>About 5 Minutes or Less: 0 (score: 0), About 10 Minutes: 1 (score: 1), About 20 Minutes: 2 (score: 2), About 30 Minutes: 3 (score: 3), About 40 Minutes: 4 (score: 4), About 50 Minutes: 5 (score: 5), More Than 1 Hour: 6 (score: 6)</t>
+  </si>
+  <si>
+    <t>Water: 0 (score: 1), Milk: 1 (score: 2), A caffeinated beverage (like coffee, tea, soda…) : 2 (score: 3), An alcoholic beverage (wine, beer, liquor…): 3 (score: 4), A beverage containing sugar like juice or caffeine free soda: 4 (score: 5), Another type of drink: 5 (score: 6), I did not drink: 6 (score: 7)</t>
+  </si>
+  <si>
+    <t>1 8-oz Glass: 1 (score: 1), 2 8-oz Glasses: 2 (score: 2), 3 8-oz Glasses: 3 (score: 3), 4 8-oz Glasses: 4 (score: 4), 5 8-oz Glasses: 5 (score: 5), 6 8-oz Glasses: 6 (score: 6), 7 8-oz Glasses: 7 (score: 7), 8 8-oz Glasses: 8 (score: 8), 9 8-oz Glasses: 9 (score: 9), 10 or More 8-oz Glasses: 10 (score: 10)</t>
+  </si>
+  <si>
+    <t>1 Serving: 1 (score: 1), 2 Servings: 2 (score: 2), 3 Servings: 3 (score: 3), 4 Serving: 4 (score: 4), 5 Servings: 5 (score: 5), 6 Servings: 6 (score: 6), 7 Servings: 7 (score: 7), 8 Servings: 8 (score: 8), 9 Servings: 9 (score: 9), 10 or More Servings: 10 (score: 10)</t>
+  </si>
+  <si>
+    <t>None: 0 (score: 0), 1: 1 (score: 1), 2: 2 (score: 2), 3: 3 (score: 3), 4: 4 (score: 4), 5: 5 (score: 5), 6: 6 (score: 6), 7: 7 (score: 7), 8: 8 (score: 8), 9: 9 (score: 9), 10: 10 (score: 10)</t>
+  </si>
+  <si>
+    <t>Just a Snack: 1 (score: 1), Continuous Snacking: 2 (score: 2), A Small Meal: 3 (score: 3), A Regular/Full Meal: 4 (score: 4), A Large Meal: 5 (score: 5)</t>
+  </si>
+  <si>
+    <t>Headache: 0 (score: 1), Back/neck/shoulder: 1 (score: 2), Arms/hands: 2 (score: 3), Feet/legs: 3 (score: 4), Stomach/bowel: 4 (score: 5), Menstrual cramps (Females only): 5 (score: 6), Other Perineal (Females only) : 6 (score: 7)</t>
+  </si>
+  <si>
+    <t>No: 0 (score: 0), Yes: 1 (score: 1)</t>
+  </si>
+  <si>
+    <t>Allergies: 0 (score: 1), Asthma or breathing difficulties: 1 (score: 2), Gastrointestinal, bowel or stomach problems : 2 (score: 3), Muscle/joint pain: 3 (score: 4), Heart racing or pounding: 4 (score: 5), Feeling faint or dizzy: 6 (score: 6), Fever/Cold: 7 (score: 7), None of the above: 8 (score: 8)</t>
+  </si>
+  <si>
+    <t>Not at all: 0 (score: 1), Mildly: 1 (score: 2), Moderately: 2 (score: 3), Severely: 3 (score: 4)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1230,8 +1296,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1278,12 +1350,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF4472C4"/>
         <bgColor theme="8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1413,7 +1479,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1485,20 +1551,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1521,6 +1575,26 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1860,34 +1934,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DC3F330-7399-DF41-9FB7-43E7ACD75EF2}">
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.6640625" style="8" customWidth="1"/>
     <col min="2" max="2" width="33.33203125" style="8" customWidth="1"/>
     <col min="3" max="3" width="21" style="8" customWidth="1"/>
     <col min="4" max="5" width="26.6640625" style="8" customWidth="1"/>
-    <col min="6" max="6" width="18" style="8" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" style="8" customWidth="1"/>
-    <col min="8" max="8" width="23.83203125" style="8" customWidth="1"/>
-    <col min="9" max="16384" width="10.83203125" style="8"/>
+    <col min="6" max="7" width="18" style="8" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" style="8" customWidth="1"/>
+    <col min="9" max="9" width="23.83203125" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="10.83203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="25" t="s">
         <v>236</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="30" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="23"/>
-    </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I1" s="23"/>
+    </row>
+    <row r="2" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1906,26 +1981,30 @@
       <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="H2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="I2" s="11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="31" t="s">
+    <row r="3" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="27" t="s">
         <v>266</v>
       </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="33"/>
-    </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="29"/>
+    </row>
+    <row r="4" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>9</v>
       </c>
@@ -1944,14 +2023,15 @@
       <c r="F4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="2"/>
+      <c r="H4" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I4" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
         <v>9</v>
       </c>
@@ -1970,14 +2050,15 @@
       <c r="F5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="G5" s="2"/>
+      <c r="H5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -1996,14 +2077,15 @@
       <c r="F6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G6" s="2"/>
+      <c r="H6" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I6" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
         <v>9</v>
       </c>
@@ -2022,14 +2104,15 @@
       <c r="F7" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="10"/>
+      <c r="H7" s="16" t="s">
         <v>231</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="I7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
@@ -2048,14 +2131,15 @@
       <c r="F8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="21" t="s">
+      <c r="G8" s="2"/>
+      <c r="H8" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I8" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
         <v>9</v>
       </c>
@@ -2074,14 +2158,15 @@
       <c r="F9" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="G9" s="10"/>
+      <c r="H9" s="16" t="s">
         <v>235</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I9" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
         <v>9</v>
       </c>
@@ -2100,14 +2185,15 @@
       <c r="F10" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G10" s="16" t="s">
+      <c r="G10" s="10"/>
+      <c r="H10" s="16" t="s">
         <v>233</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I10" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="10" t="s">
         <v>9</v>
       </c>
@@ -2126,14 +2212,15 @@
       <c r="F11" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="G11" s="10"/>
+      <c r="H11" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I11" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
         <v>9</v>
       </c>
@@ -2152,14 +2239,15 @@
       <c r="F12" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="16" t="s">
+      <c r="G12" s="10"/>
+      <c r="H12" s="16" t="s">
         <v>232</v>
       </c>
-      <c r="H12" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I12" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
         <v>9</v>
       </c>
@@ -2178,14 +2266,15 @@
       <c r="F13" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="10"/>
+      <c r="H13" s="16" t="s">
         <v>257</v>
       </c>
-      <c r="H13" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I13" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
         <v>9</v>
       </c>
@@ -2204,14 +2293,15 @@
       <c r="F14" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="16" t="s">
+      <c r="G14" s="10"/>
+      <c r="H14" s="16" t="s">
         <v>259</v>
       </c>
-      <c r="H14" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I14" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
         <v>9</v>
       </c>
@@ -2230,14 +2320,15 @@
       <c r="F15" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="16" t="s">
+      <c r="G15" s="10"/>
+      <c r="H15" s="16" t="s">
         <v>261</v>
       </c>
-      <c r="H15" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I15" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
         <v>9</v>
       </c>
@@ -2256,14 +2347,15 @@
       <c r="F16" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="10"/>
+      <c r="H16" t="s">
         <v>263</v>
       </c>
-      <c r="H16" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I16" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="10" t="s">
         <v>9</v>
       </c>
@@ -2282,26 +2374,28 @@
       <c r="F17" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G17" s="16" t="s">
+      <c r="G17" s="10"/>
+      <c r="H17" s="16" t="s">
         <v>265</v>
       </c>
-      <c r="H17" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="31" t="s">
+      <c r="I17" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="27" t="s">
         <v>239</v>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="33"/>
-    </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="29"/>
+    </row>
+    <row r="19" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="10" t="s">
         <v>9</v>
       </c>
@@ -2320,14 +2414,15 @@
       <c r="F19" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G19" s="16" t="s">
+      <c r="G19" s="10"/>
+      <c r="H19" s="16" t="s">
         <v>231</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I19" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
         <v>9</v>
       </c>
@@ -2346,14 +2441,15 @@
       <c r="F20" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="10"/>
+      <c r="H20" t="s">
         <v>241</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I20" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="10" t="s">
         <v>9</v>
       </c>
@@ -2372,14 +2468,15 @@
       <c r="F21" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="10"/>
+      <c r="H21" t="s">
         <v>243</v>
       </c>
-      <c r="H21" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I21" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="10" t="s">
         <v>9</v>
       </c>
@@ -2398,14 +2495,15 @@
       <c r="F22" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="10"/>
+      <c r="H22" t="s">
         <v>255</v>
       </c>
-      <c r="H22" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I22" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="10" t="s">
         <v>9</v>
       </c>
@@ -2424,14 +2522,15 @@
       <c r="F23" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" s="10"/>
+      <c r="H23" t="s">
         <v>246</v>
       </c>
-      <c r="H23" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I23" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="10" t="s">
         <v>9</v>
       </c>
@@ -2450,14 +2549,15 @@
       <c r="F24" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="10"/>
+      <c r="H24" t="s">
         <v>248</v>
       </c>
-      <c r="H24" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I24" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="10" t="s">
         <v>9</v>
       </c>
@@ -2476,14 +2576,15 @@
       <c r="F25" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="10"/>
+      <c r="H25" t="s">
         <v>250</v>
       </c>
-      <c r="H25" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I25" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="10" t="s">
         <v>9</v>
       </c>
@@ -2502,14 +2603,15 @@
       <c r="F26" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" s="10"/>
+      <c r="H26" t="s">
         <v>252</v>
       </c>
-      <c r="H26" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I26" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="10" t="s">
         <v>9</v>
       </c>
@@ -2528,27 +2630,29 @@
       <c r="F27" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" s="10"/>
+      <c r="H27" t="s">
         <v>254</v>
       </c>
-      <c r="H27" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="34" t="s">
+      <c r="I27" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="35"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="35"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="35"/>
-      <c r="H28" s="36"/>
-    </row>
-    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="25" t="s">
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="32"/>
+    </row>
+    <row r="29" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="33" t="s">
         <v>18</v>
       </c>
       <c r="B29" s="23"/>
@@ -2557,9 +2661,10 @@
       <c r="E29" s="23"/>
       <c r="F29" s="23"/>
       <c r="G29" s="23"/>
-      <c r="H29" s="24"/>
-    </row>
-    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H29" s="23"/>
+      <c r="I29" s="24"/>
+    </row>
+    <row r="30" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
         <v>19</v>
       </c>
@@ -2576,14 +2681,17 @@
       <c r="F30" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G30" s="13" t="s">
+      <c r="G30" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="H30" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="H30" s="15" t="s">
+      <c r="I30" s="15" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
         <v>19</v>
       </c>
@@ -2602,14 +2710,17 @@
       <c r="F31" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G31" s="3" t="s">
+      <c r="G31" s="39" t="s">
+        <v>268</v>
+      </c>
+      <c r="H31" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H31" s="14" t="s">
+      <c r="I31" s="14" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
         <v>19</v>
       </c>
@@ -2628,12 +2739,15 @@
       <c r="F32" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G32" s="3" t="s">
+      <c r="G32" s="39" t="s">
+        <v>268</v>
+      </c>
+      <c r="H32" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H32" s="6"/>
-    </row>
-    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I32" s="6"/>
+    </row>
+    <row r="33" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
         <v>19</v>
       </c>
@@ -2652,12 +2766,15 @@
       <c r="F33" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="G33" s="40" t="s">
+        <v>268</v>
+      </c>
+      <c r="H33" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H33" s="6"/>
-    </row>
-    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I33" s="6"/>
+    </row>
+    <row r="34" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
         <v>19</v>
       </c>
@@ -2676,12 +2793,15 @@
       <c r="F34" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="G34" s="40" t="s">
+        <v>268</v>
+      </c>
+      <c r="H34" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="H34" s="6"/>
-    </row>
-    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I34" s="6"/>
+    </row>
+    <row r="35" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
         <v>19</v>
       </c>
@@ -2700,12 +2820,15 @@
       <c r="F35" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G35" s="3" t="s">
+      <c r="G35" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H35" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="H35" s="6"/>
-    </row>
-    <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I35" s="6"/>
+    </row>
+    <row r="36" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
         <v>19</v>
       </c>
@@ -2724,13 +2847,16 @@
       <c r="F36" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="G36" s="3" t="s">
+      <c r="G36" s="40" t="s">
+        <v>270</v>
+      </c>
+      <c r="H36" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="H36" s="6"/>
-    </row>
-    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="25" t="s">
+      <c r="I36" s="6"/>
+    </row>
+    <row r="37" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="33" t="s">
         <v>48</v>
       </c>
       <c r="B37" s="23"/>
@@ -2739,9 +2865,10 @@
       <c r="E37" s="23"/>
       <c r="F37" s="23"/>
       <c r="G37" s="23"/>
-      <c r="H37" s="24"/>
-    </row>
-    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H37" s="23"/>
+      <c r="I37" s="24"/>
+    </row>
+    <row r="38" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
         <v>49</v>
       </c>
@@ -2758,12 +2885,15 @@
       <c r="F38" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G38" s="3" t="s">
+      <c r="G38" s="40" t="s">
+        <v>271</v>
+      </c>
+      <c r="H38" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="H38" s="3"/>
-    </row>
-    <row r="39" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I38" s="3"/>
+    </row>
+    <row r="39" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
         <v>49</v>
       </c>
@@ -2782,14 +2912,17 @@
       <c r="F39" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="G39" s="3" t="s">
+      <c r="G39" s="40" t="s">
+        <v>272</v>
+      </c>
+      <c r="H39" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="H39" s="3" t="s">
+      <c r="I39" s="3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
         <v>49</v>
       </c>
@@ -2808,14 +2941,17 @@
       <c r="F40" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G40" s="3" t="s">
+      <c r="G40" s="40" t="s">
+        <v>273</v>
+      </c>
+      <c r="H40" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="I40" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
         <v>49</v>
       </c>
@@ -2834,14 +2970,17 @@
       <c r="F41" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G41" s="3" t="s">
+      <c r="G41" s="40" t="s">
+        <v>274</v>
+      </c>
+      <c r="H41" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H41" s="3" t="s">
+      <c r="I41" s="3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>49</v>
       </c>
@@ -2858,15 +2997,18 @@
       <c r="F42" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="G42" s="3" t="s">
+      <c r="G42" s="40" t="s">
+        <v>275</v>
+      </c>
+      <c r="H42" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="H42" s="3" t="s">
+      <c r="I42" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="26" t="s">
+    <row r="43" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="34" t="s">
         <v>78</v>
       </c>
       <c r="B43" s="23"/>
@@ -2875,9 +3017,10 @@
       <c r="E43" s="23"/>
       <c r="F43" s="23"/>
       <c r="G43" s="23"/>
-      <c r="H43" s="24"/>
-    </row>
-    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H43" s="23"/>
+      <c r="I43" s="24"/>
+    </row>
+    <row r="44" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
         <v>49</v>
       </c>
@@ -2896,13 +3039,16 @@
       <c r="F44" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="G44" s="10" t="s">
+      <c r="G44" s="40" t="s">
+        <v>276</v>
+      </c>
+      <c r="H44" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="H44" s="6"/>
-    </row>
-    <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="26" t="s">
+      <c r="I44" s="6"/>
+    </row>
+    <row r="45" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="34" t="s">
         <v>84</v>
       </c>
       <c r="B45" s="23"/>
@@ -2911,9 +3057,10 @@
       <c r="E45" s="23"/>
       <c r="F45" s="23"/>
       <c r="G45" s="23"/>
-      <c r="H45" s="24"/>
-    </row>
-    <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H45" s="23"/>
+      <c r="I45" s="24"/>
+    </row>
+    <row r="46" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>85</v>
       </c>
@@ -2930,12 +3077,15 @@
       <c r="F46" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="G46" s="3" t="s">
+      <c r="G46" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H46" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H46" s="6"/>
-    </row>
-    <row r="47" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I46" s="6"/>
+    </row>
+    <row r="47" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
         <v>85</v>
       </c>
@@ -2952,12 +3102,15 @@
       <c r="F47" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="G47" s="3" t="s">
+      <c r="G47" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H47" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H47" s="6"/>
-    </row>
-    <row r="48" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I47" s="6"/>
+    </row>
+    <row r="48" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
         <v>85</v>
       </c>
@@ -2974,12 +3127,15 @@
       <c r="F48" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="G48" s="3" t="s">
+      <c r="G48" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H48" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="H48" s="6"/>
-    </row>
-    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I48" s="6"/>
+    </row>
+    <row r="49" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="6" t="s">
         <v>85</v>
       </c>
@@ -2996,13 +3152,16 @@
       <c r="F49" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="G49" s="3" t="s">
+      <c r="G49" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H49" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="H49" s="6"/>
-    </row>
-    <row r="50" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="27" t="s">
+      <c r="I49" s="6"/>
+    </row>
+    <row r="50" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="35" t="s">
         <v>102</v>
       </c>
       <c r="B50" s="23"/>
@@ -3011,9 +3170,10 @@
       <c r="E50" s="23"/>
       <c r="F50" s="23"/>
       <c r="G50" s="23"/>
-      <c r="H50" s="24"/>
-    </row>
-    <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H50" s="23"/>
+      <c r="I50" s="24"/>
+    </row>
+    <row r="51" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
         <v>85</v>
       </c>
@@ -3030,14 +3190,17 @@
       <c r="F51" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="G51" s="3" t="s">
+      <c r="G51" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H51" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="H51" s="3" t="s">
+      <c r="I51" s="3" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
         <v>85</v>
       </c>
@@ -3054,14 +3217,17 @@
       <c r="F52" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="G52" s="3" t="s">
+      <c r="G52" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H52" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="H52" s="3" t="s">
+      <c r="I52" s="3" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="22" t="s">
         <v>113</v>
       </c>
@@ -3071,9 +3237,10 @@
       <c r="E53" s="23"/>
       <c r="F53" s="23"/>
       <c r="G53" s="23"/>
-      <c r="H53" s="24"/>
-    </row>
-    <row r="54" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H53" s="23"/>
+      <c r="I53" s="24"/>
+    </row>
+    <row r="54" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="6" t="s">
         <v>114</v>
       </c>
@@ -3090,14 +3257,17 @@
       <c r="F54" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="G54" s="3" t="s">
+      <c r="G54" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="H54" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="H54" s="3" t="s">
+      <c r="I54" s="3" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="6" t="s">
         <v>114</v>
       </c>
@@ -3114,12 +3284,15 @@
       <c r="F55" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="G55" s="3" t="s">
+      <c r="G55" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H55" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="H55" s="6"/>
-    </row>
-    <row r="56" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I55" s="6"/>
+    </row>
+    <row r="56" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
         <v>114</v>
       </c>
@@ -3136,14 +3309,17 @@
       <c r="F56" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="G56" s="3" t="s">
+      <c r="G56" s="40" t="s">
+        <v>277</v>
+      </c>
+      <c r="H56" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="H56" s="3" t="s">
+      <c r="I56" s="3" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
         <v>114</v>
       </c>
@@ -3160,15 +3336,18 @@
       <c r="F57" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="G57" s="3" t="s">
+      <c r="G57" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H57" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="H57" s="3" t="s">
+      <c r="I57" s="3" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="25" t="s">
+    <row r="58" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="33" t="s">
         <v>134</v>
       </c>
       <c r="B58" s="23"/>
@@ -3177,9 +3356,10 @@
       <c r="E58" s="23"/>
       <c r="F58" s="23"/>
       <c r="G58" s="23"/>
-      <c r="H58" s="24"/>
-    </row>
-    <row r="59" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H58" s="23"/>
+      <c r="I58" s="24"/>
+    </row>
+    <row r="59" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="6" t="s">
         <v>135</v>
       </c>
@@ -3196,14 +3376,17 @@
       <c r="F59" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="G59" s="3" t="s">
+      <c r="G59" s="40" t="s">
+        <v>278</v>
+      </c>
+      <c r="H59" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="H59" s="3" t="s">
+      <c r="I59" s="3" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
         <v>135</v>
       </c>
@@ -3222,12 +3405,15 @@
       <c r="F60" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="G60" s="3" t="s">
+      <c r="G60" s="40" t="s">
+        <v>279</v>
+      </c>
+      <c r="H60" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="H60" s="6"/>
-    </row>
-    <row r="61" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I60" s="6"/>
+    </row>
+    <row r="61" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="6" t="s">
         <v>135</v>
       </c>
@@ -3246,12 +3432,15 @@
       <c r="F61" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="G61" s="3" t="s">
+      <c r="G61" s="40" t="s">
+        <v>279</v>
+      </c>
+      <c r="H61" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="H61" s="6"/>
-    </row>
-    <row r="62" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I61" s="6"/>
+    </row>
+    <row r="62" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="6" t="s">
         <v>135</v>
       </c>
@@ -3270,12 +3459,15 @@
       <c r="F62" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="G62" s="6" t="s">
+      <c r="G62" s="40" t="s">
+        <v>279</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="H62" s="6"/>
-    </row>
-    <row r="63" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I62" s="6"/>
+    </row>
+    <row r="63" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="22" t="s">
         <v>154</v>
       </c>
@@ -3285,9 +3477,10 @@
       <c r="E63" s="23"/>
       <c r="F63" s="23"/>
       <c r="G63" s="23"/>
-      <c r="H63" s="24"/>
-    </row>
-    <row r="64" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H63" s="23"/>
+      <c r="I63" s="24"/>
+    </row>
+    <row r="64" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
         <v>155</v>
       </c>
@@ -3304,14 +3497,17 @@
       <c r="F64" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="G64" s="3" t="s">
+      <c r="G64" s="40" t="s">
+        <v>280</v>
+      </c>
+      <c r="H64" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="H64" s="3" t="s">
+      <c r="I64" s="3" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>155</v>
       </c>
@@ -3330,12 +3526,15 @@
       <c r="F65" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="G65" s="3" t="s">
+      <c r="G65" s="40" t="s">
+        <v>281</v>
+      </c>
+      <c r="H65" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="H65" s="6"/>
-    </row>
-    <row r="66" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I65" s="6"/>
+    </row>
+    <row r="66" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
         <v>155</v>
       </c>
@@ -3354,14 +3553,17 @@
       <c r="F66" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="G66" s="3" t="s">
+      <c r="G66" s="40" t="s">
+        <v>282</v>
+      </c>
+      <c r="H66" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="H66" s="3" t="s">
+      <c r="I66" s="3" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
         <v>155</v>
       </c>
@@ -3378,12 +3580,15 @@
       <c r="F67" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="G67" s="3" t="s">
+      <c r="G67" s="40" t="s">
+        <v>283</v>
+      </c>
+      <c r="H67" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="H67" s="6"/>
-    </row>
-    <row r="68" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I67" s="6"/>
+    </row>
+    <row r="68" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>155</v>
       </c>
@@ -3402,12 +3607,15 @@
       <c r="F68" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="G68" s="3" t="s">
+      <c r="G68" s="40" t="s">
+        <v>284</v>
+      </c>
+      <c r="H68" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="H68" s="6"/>
-    </row>
-    <row r="69" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I68" s="6"/>
+    </row>
+    <row r="69" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="22" t="s">
         <v>181</v>
       </c>
@@ -3417,9 +3625,10 @@
       <c r="E69" s="23"/>
       <c r="F69" s="23"/>
       <c r="G69" s="23"/>
-      <c r="H69" s="24"/>
-    </row>
-    <row r="70" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H69" s="23"/>
+      <c r="I69" s="24"/>
+    </row>
+    <row r="70" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="22" t="s">
         <v>183</v>
       </c>
@@ -3429,10 +3638,11 @@
       <c r="E70" s="23"/>
       <c r="F70" s="23"/>
       <c r="G70" s="23"/>
-      <c r="H70" s="24"/>
-    </row>
-    <row r="71" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="25" t="s">
+      <c r="H70" s="23"/>
+      <c r="I70" s="24"/>
+    </row>
+    <row r="71" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="33" t="s">
         <v>184</v>
       </c>
       <c r="B71" s="23"/>
@@ -3441,9 +3651,10 @@
       <c r="E71" s="23"/>
       <c r="F71" s="23"/>
       <c r="G71" s="23"/>
-      <c r="H71" s="24"/>
-    </row>
-    <row r="72" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H71" s="23"/>
+      <c r="I71" s="24"/>
+    </row>
+    <row r="72" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
         <v>185</v>
       </c>
@@ -3460,12 +3671,15 @@
       <c r="F72" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="G72" s="3" t="s">
+      <c r="G72" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H72" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="H72" s="6"/>
-    </row>
-    <row r="73" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I72" s="6"/>
+    </row>
+    <row r="73" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="6" t="s">
         <v>185</v>
       </c>
@@ -3484,12 +3698,15 @@
       <c r="F73" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="G73" s="3" t="s">
+      <c r="G73" s="40" t="s">
+        <v>285</v>
+      </c>
+      <c r="H73" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="H73" s="3"/>
-    </row>
-    <row r="74" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I73" s="3"/>
+    </row>
+    <row r="74" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="6" t="s">
         <v>185</v>
       </c>
@@ -3506,12 +3723,15 @@
       <c r="F74" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="G74" s="3" t="s">
+      <c r="G74" s="40" t="s">
+        <v>286</v>
+      </c>
+      <c r="H74" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="H74" s="6"/>
-    </row>
-    <row r="75" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I74" s="6"/>
+    </row>
+    <row r="75" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="6" t="s">
         <v>185</v>
       </c>
@@ -3530,12 +3750,15 @@
       <c r="F75" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="G75" s="3" t="s">
+      <c r="G75" s="40" t="s">
+        <v>285</v>
+      </c>
+      <c r="H75" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="H75" s="3"/>
-    </row>
-    <row r="76" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I75" s="3"/>
+    </row>
+    <row r="76" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="6" t="s">
         <v>185</v>
       </c>
@@ -3554,12 +3777,15 @@
       <c r="F76" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="G76" s="3" t="s">
+      <c r="G76" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H76" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="H76" s="6"/>
-    </row>
-    <row r="77" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I76" s="6"/>
+    </row>
+    <row r="77" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="22" t="s">
         <v>208</v>
       </c>
@@ -3569,10 +3795,11 @@
       <c r="E77" s="23"/>
       <c r="F77" s="23"/>
       <c r="G77" s="23"/>
-      <c r="H77" s="24"/>
-    </row>
-    <row r="78" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="26" t="s">
+      <c r="H77" s="23"/>
+      <c r="I77" s="24"/>
+    </row>
+    <row r="78" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="34" t="s">
         <v>210</v>
       </c>
       <c r="B78" s="23"/>
@@ -3581,9 +3808,10 @@
       <c r="E78" s="23"/>
       <c r="F78" s="23"/>
       <c r="G78" s="23"/>
-      <c r="H78" s="24"/>
-    </row>
-    <row r="79" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H78" s="23"/>
+      <c r="I78" s="24"/>
+    </row>
+    <row r="79" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="6" t="s">
         <v>211</v>
       </c>
@@ -3600,12 +3828,15 @@
       <c r="F79" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="G79" s="3" t="s">
+      <c r="G79" s="40" t="s">
+        <v>269</v>
+      </c>
+      <c r="H79" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="H79" s="6"/>
-    </row>
-    <row r="80" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I79" s="6"/>
+    </row>
+    <row r="80" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="6" t="s">
         <v>211</v>
       </c>
@@ -3622,12 +3853,15 @@
       <c r="F80" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="G80" s="3" t="s">
+      <c r="G80" s="40" t="s">
+        <v>287</v>
+      </c>
+      <c r="H80" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="H80" s="6"/>
-    </row>
-    <row r="81" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I80" s="6"/>
+    </row>
+    <row r="81" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="6" t="s">
         <v>211</v>
       </c>
@@ -3646,13 +3880,16 @@
       <c r="F81" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="G81" s="10" t="s">
+      <c r="G81" s="40" t="s">
+        <v>288</v>
+      </c>
+      <c r="H81" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="H81" s="6"/>
-    </row>
-    <row r="82" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="27" t="s">
+      <c r="I81" s="6"/>
+    </row>
+    <row r="82" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="35" t="s">
         <v>224</v>
       </c>
       <c r="B82" s="23"/>
@@ -3661,9 +3898,10 @@
       <c r="E82" s="23"/>
       <c r="F82" s="23"/>
       <c r="G82" s="23"/>
-      <c r="H82" s="24"/>
-    </row>
-    <row r="83" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H82" s="23"/>
+      <c r="I82" s="24"/>
+    </row>
+    <row r="83" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="22" t="s">
         <v>225</v>
       </c>
@@ -3673,30 +3911,31 @@
       <c r="E83" s="23"/>
       <c r="F83" s="23"/>
       <c r="G83" s="23"/>
-      <c r="H83" s="24"/>
+      <c r="H83" s="23"/>
+      <c r="I83" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A63:H63"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A50:H50"/>
-    <mergeCell ref="A53:H53"/>
-    <mergeCell ref="A58:H58"/>
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A83:H83"/>
-    <mergeCell ref="A69:H69"/>
-    <mergeCell ref="A70:H70"/>
-    <mergeCell ref="A71:H71"/>
-    <mergeCell ref="A77:H77"/>
-    <mergeCell ref="A78:H78"/>
-    <mergeCell ref="A82:H82"/>
+    <mergeCell ref="A83:I83"/>
+    <mergeCell ref="A69:I69"/>
+    <mergeCell ref="A70:I70"/>
+    <mergeCell ref="A71:I71"/>
+    <mergeCell ref="A77:I77"/>
+    <mergeCell ref="A78:I78"/>
+    <mergeCell ref="A82:I82"/>
+    <mergeCell ref="A63:I63"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A53:I53"/>
+    <mergeCell ref="A58:I58"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>